<commit_message>
feat: implement 18-node n8n workflow, direct POS checkout, and resilient UI error handling
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -559,7 +559,7 @@
         <v>40</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F2" s="4" t="n">
         <v>2</v>
@@ -590,7 +590,7 @@
         <v>38</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F3" s="4" t="n">
         <v>2</v>
@@ -621,7 +621,7 @@
         <v>38</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>2</v>
@@ -652,7 +652,7 @@
         <v>39</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>2</v>
@@ -671,7 +671,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Bleu Impérial</t>
+          <t>Bleu Imperial</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -683,7 +683,7 @@
         <v>38</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>2</v>
@@ -714,7 +714,7 @@
         <v>10</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>5</v>
@@ -807,7 +807,7 @@
         <v>18</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>2</v>
@@ -860,7 +860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1090,6 +1090,651 @@
       <c r="I5" t="inlineStr">
         <is>
           <t>Total value is $20.00, which is under $100, and stock (18) is sufficient for the requested quantity (2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ORD-DE16B07F</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Walk-In Customer</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Bleu Impérial</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Blue 100ml</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>76</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:52:58.573117+00:00</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Total value is $76.00, which is below the $100 threshold, and stock (10) is sufficient for the requested quantity (2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ORD-C2C7408B</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Demo Cashier</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Basic Shirt</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>20</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:56:56.755312+00:00</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>POS Auto-fulfilled (&lt;$100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ORD-451DFCBA</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Walk-In Customer</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Chic Oriental</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Gold 100ml</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>39</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:03:04.046032+00:00</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Total value is $39.00, which is under the $100 threshold, and stock (10) is sufficient for the requested quantity (1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ORD-C32063F7</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Walk-In Customer</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Premium Shirt</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>54</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:06:59.940141+00:00</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>POS Auto-fulfilled (&lt;$100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ORD-9003186C</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Walk-In Customer</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Bleu Imperial</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Blue 100ml</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>38</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:11:20.543003+00:00</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>POS Auto-fulfilled (&lt;$100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ORD-D634B216</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Jane Smith</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>shirt</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>10</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:14:25.726103+00:00</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Total value is $10.00, which is under $100, and stock (20) is sufficient for the requested quantity (1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ORD-503345A7</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Jane Smith</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>shirt</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>10</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:14:27.564858+00:00</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Total value is $10.00 (&lt; $100) and stock (20) is sufficient for the requested quantity (1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ORD-E31B4368</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Walk-In Customer</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Chic Oriental</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Gold 100ml</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>39</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:19:34.703362+00:00</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>POS Auto-fulfilled (&lt;$100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ORD-12944DB3</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Walk-In Customer</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Chic Oriental</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Gold 100ml</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>39</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:19:59.586613+00:00</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>POS Auto-fulfilled (&lt;$100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ORD-DC3CFD8F</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Walk-In Customer</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Cherry Delice</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Red 100ml</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>38</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:22:58.982616+00:00</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>POS Auto-fulfilled (&lt;$100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ORD-03E46541</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Walk-In Customer</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Yes I Am The King Le</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Black 100ml</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>38</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:23:35.782497+00:00</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>POS Auto-fulfilled (&lt;$100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ORD-A167332A</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Walk-In Customer</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Cherry Delice</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Red 100ml</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>38</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:24:50.566771+00:00</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>POS Auto-fulfilled (&lt;$100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ORD-951AE1EF</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Walk-In Customer</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Yes I Am The Queen</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Pink 100ml</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>40</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:28:40.029617+00:00</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>POS Auto-fulfilled (&lt;$100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ORD-E8074C23</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Walk-In Customer</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Bleu Imperial</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Blue 100ml</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>38</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:29:08.160373+00:00</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>POS Auto-fulfilled (&lt;$100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ORD-1AA07BE0</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Walk-In Customer</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>shirt</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>blue</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>10</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:32:19.556493+00:00</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Total value is $10.00, which is under the $100 threshold, and stock (19) is sufficient for the requested quantity (1).</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1527,6 +2172,1350 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LOG-847EB2E7</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:52:58.573117+00:00</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ORD-DE16B07F</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Total value is $76.00, which is below the $100 threshold, and stock (10) is sufficient for the requested quantity (2).</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LOG-4AC40926</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-10-04T09:56:56.755312+00:00</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ORD-C2C7408B</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>POS cart checkout fulfilled ($20.00)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LOG-44FE7D2E</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:03:04.046032+00:00</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ORD-451DFCBA</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Total value is $39.00, which is under the $100 threshold, and stock (10) is sufficient for the requested quantity (1).</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LOG-C2781159</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:06:04.158624+00:00</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>owner_escalation</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ORD-C765EDF7</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>High value cart order ($130.00 &gt;= $100)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LOG-04E535CA</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:06:34.269134+00:00</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>owner_escalation</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ORD-BBC95CAC</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>High value cart order ($126.00 &gt;= $100)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>LOG-9A4985D5</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:06:59.940141+00:00</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ORD-C32063F7</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>POS cart checkout fulfilled ($54.00)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LOG-8537FEA6</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:08:31.909994+00:00</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>clarification_requested</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ORD-328E3BB0</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Product not found or quantity unclear</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>LOG-425D1118</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:08:33.373367+00:00</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>clarification_requested</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ORD-AA04D33F</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Product not found or quantity unclear</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>LOG-F39BC38A</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:09:16.326534+00:00</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>clarification_requested</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>ORD-A2793934</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Product not found or quantity unclear</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>LOG-2085687B</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:09:18.883909+00:00</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>clarification_requested</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ORD-B15821A0</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Product not found or quantity unclear</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>LOG-F8C22FE2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:09:21.230219+00:00</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>order_rejected</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ORD-3E16474B</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Requested quantity (1000) exceeds available stock (15) for Basic Shirt Red. No alternative variant or product has sufficient stock to fulfill the requested quantity.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>LOG-1B8D0F99</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:11:03.533461+00:00</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>clarification_requested</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ORD-313D615B</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Product not found or quantity unclear</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>LOG-D07E8493</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:11:20.543003+00:00</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>ORD-9003186C</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>POS cart checkout fulfilled ($38.00)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>LOG-9DECA987</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:11:32.640717+00:00</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>clarification_requested</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>ORD-2B8B2AFA</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Product not found or quantity unclear</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>LOG-F8E2BAFE</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:11:35.066972+00:00</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>alternative_suggested</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ORD-5943A533</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Requested quantity (1000) exceeds available stock (15) for Basic Shirt in Red. Other Basic Shirt variants (Black, White) and Premium Shirt variants are available in inventory, so an alternative can be suggested.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>LOG-7FCDF39A</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:11:46.927836+00:00</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>alternative_suggested</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ORD-F9498780</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Requested quantity (500) exceeds available stock (10) for 'Yes I Am The Queen' Pink 100ml. No other variant of the same product is available, but similar products in the same category (Beauty) have sufficient stock to fulfill the requested quantity.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>LOG-DA12CD87</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:11:51.293805+00:00</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>alternative_suggested</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ORD-72B49418</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Requested quantity (500) exceeds available stock (15) for Basic Shirt Red. Alternative variants of Basic Shirt are available in sufficient quantity to fulfill the order.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>LOG-BBD0BA31</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:11:55.899996+00:00</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>alternative_suggested</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ORD-4FC1CFCF</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Requested quantity (500) exceeds available stock (15) for Basic Shirt Red. Alternative Basic Shirt variants are available in inventory.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>LOG-04E542CA</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:12:24.540525+00:00</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>owner_escalation</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ORD-EB46A11A</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>High value cart order ($183.00 &gt;= $100)</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>LOG-02D8D984</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:12:24.299511+00:00</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>order_rejected</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ORD-EDEDA04E</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Requested quantity (1000) exceeds available stock (15) and total store inventory cannot fulfill the order. No alternative variant has sufficient stock to cover the requested quantity.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LOG-30E9E0CE</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:12:40.858848+00:00</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>clarification_requested</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>ORD-06A0893A</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Product not found or quantity unclear</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>LOG-3BA85C36</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:12:44.267829+00:00</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>order_rejected</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>ORD-B882B5C3</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Requested quantity (1000) far exceeds available stock (15) and total store inventory cannot fulfill it; also exceeds the 500-unit threshold for rejection.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>LOG-E3F8C9BE</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:13:16.933871+00:00</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>order_rejected</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>ORD-C9A493A8</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Requested quantity (1000) exceeds available stock (15) and total store inventory for this product (53 across all variants). Per rule 4, reject when stock is insufficient and total store inventory cannot fulfill the requested quantity.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>LOG-EA994133</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:13:41.461266+00:00</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>clarification_requested</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>ORD-BBC599F5</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Product not found or quantity unclear</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>LOG-0B512B6C</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:14:07.223297+00:00</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>clarification_requested</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>ORD-C507A96A</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Product not found or quantity unclear</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>LOG-4C4EBA72</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:14:08.917563+00:00</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>clarification_requested</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>ORD-9C104C1B</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Product not found or quantity unclear</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>LOG-F7BA2F22</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:14:25.726103+00:00</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>ORD-D634B216</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Total value is $10.00, which is under $100, and stock (20) is sufficient for the requested quantity (1).</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>LOG-8FCE7365</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:14:27.564858+00:00</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>ORD-503345A7</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Total value is $10.00 (&lt; $100) and stock (20) is sufficient for the requested quantity (1).</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>LOG-FA84B040</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:19:34.703362+00:00</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>ORD-E31B4368</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>POS cart checkout fulfilled ($39.00)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>LOG-1D0ADC10</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:19:59.586613+00:00</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>ORD-12944DB3</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>POS cart checkout fulfilled ($39.00)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>LOG-141A4FFD</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:22:28.738715+00:00</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>clarification_requested</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>ORD-14E9A5AB</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Product not found or quantity unclear</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LOG-2B4FBF00</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:22:37.653054+00:00</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>order_rejected</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>ORD-802711C4</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Requested quantity (1000) exceeds available stock (15) and total store inventory for this product (52 across all variants), so the order cannot be fulfilled.</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>LOG-C15AAB37</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:22:58.982616+00:00</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>ORD-DC3CFD8F</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>POS cart checkout fulfilled ($38.00)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>LOG-A3A09672</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:23:35.782497+00:00</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ORD-03E46541</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>POS cart checkout fulfilled ($38.00)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>LOG-EA1BBE9A</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:24:50.566771+00:00</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>ORD-A167332A</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>POS cart checkout fulfilled ($38.00)</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>LOG-81E1668C</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:28:40.029617+00:00</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>ORD-951AE1EF</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>POS cart checkout fulfilled ($40.00)</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>LOG-FFF1EB17</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:29:08.160373+00:00</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>ORD-E8074C23</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>POS cart checkout fulfilled ($38.00)</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>LOG-C49EBA6D</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:29:30.405781+00:00</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>owner_escalation</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ORD-8BF10EA1</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>High value cart order ($152.00 &gt;= $100)</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>LOG-288E0F9F</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:31:14.005589+00:00</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>clarification_requested</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ORD-8884A6FA</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Product not found or quantity unclear</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>LOG-EAFACB0D</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:31:45.076823+00:00</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>order_rejected</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>ORD-DD68843A</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Requested quantity of 1000 units exceeds available stock (19 units) and total store inventory for this product (52 units across all variants), and the quantity is far beyond any feasible fulfillment threshold.</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>LOG-2BC05A6D</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:31:50.317168+00:00</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>order_rejected</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>ORD-A8991EE4</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Requested quantity (1000) far exceeds available stock (19) and total store inventory cannot fulfill the order. No alternative can cover the requested quantity.</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>LOG-AB0459AD</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-10-04T10:32:19.556493+00:00</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>order_approved</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ORD-1AA07BE0</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Total value is $10.00, which is under the $100 threshold, and stock (19) is sufficient for the requested quantity (1).</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>